<commit_message>
Primer: hostname, domain, FQDN and DNS side by side
Adds a four-row block to the Basics sheet showing the same real name
split into hostname, domain and FQDN, with DNS explained as the lookup
service the FQDN comes from, plus the quick test and which rule pairs
check each way a CI may store the name.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UaiSzs85tKmfaeLA1rAxsP
</commit_message>
<xml_diff>
--- a/stories/qualys-ci-lookup-rules/Qualys CI Lookup Rules - Plain English Primer.xlsx
+++ b/stories/qualys-ci-lookup-rules/Qualys CI Lookup Rules - Plain English Primer.xlsx
@@ -693,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1156,7 +1156,143 @@
         </is>
       </c>
     </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Hostname vs domain vs FQDN vs DNS - the same machine, four angles</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Take the real name from the payload: ah-1047132-001.sdi.corp.bankofamerica.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Piece</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Analogy</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Hostname</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>ah-1047132-001</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>The machine's own short name. Unique only inside its domain: another ah-1047132-001 can exist in hk.baml.com. No dots.</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>First name</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>sdi.corp.bankofamerica.com</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>The area the name belongs to.</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Surname + address</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>FQDN</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>ah-1047132-001.sdi.corp.bankofamerica.com</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Hostname + domain. "Fully qualified" = nothing missing, so it is unique everywhere. Has dots.</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>Full name on an envelope</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>DNS</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>(not a name)</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="inlineStr">
+        <is>
+          <t>The phone book of the network: it translates names to IP addresses and back. Qualys asks DNS "who is 171.128.225.96?", DNS answers with the FQDN, and Qualys puts that answer in the payload field it calls DNS. So the DNS field holds an FQDN (occasionally just a hostname, when the phone book only knows the short name).</t>
+        </is>
+      </c>
+      <c r="D32" s="9" t="inlineStr">
+        <is>
+          <t>The phone book</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="44" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Quick test: no dots = hostname; dots = FQDN; "DNS" = where the FQDN came from. The rules check every way a CI may have stored the name: the FQDN in the fqdn field (250/260), the hostname in name with the domain in dns_domain (300/310), the hostname alone (400/410), the whole FQDN typed into name (450/850).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A26:D26"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>